<commit_message>
Fix feature 6: 휴비스쌤 correction uses bCODE, not 병록번호
휴비스쌤 파일에 병록번호가 없고 bCODE만 존재하는 실제 구조 반영

- _build_pers_no(): 성별+출생연도+출생월 → 개인번호(M93.05) 재조합 헬퍼 추가
- _read_hubis_fix(): mg_donor_info 컬럼 구조 파싱, 1행 skip, bCODE 기준으로 변경
- run_update_collection_log(): 휴비스쌤=bCODE+개인번호 재조합, 슈프림=병록번호+컬럼 덮어쓰기로 분기
- generate_sample_data.py: 휴비스쌤 샘플을 mg_donor_info 실제 형식으로 수정

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/hubis_샘플.xlsx
+++ b/sample_data/hubis_샘플.xlsx
@@ -14,12 +14,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>식별코드</t>
-  </si>
-  <si>
-    <t>성별구분</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+  <si>
+    <t>mg_donor_info:KBN_DONOR</t>
+  </si>
+  <si>
+    <t>mg_donor_info:SEX</t>
+  </si>
+  <si>
+    <t>mg_donor_info:BIRTH_YEAR</t>
+  </si>
+  <si>
+    <t>mg_donor_info:BIRTH_MONTH</t>
+  </si>
+  <si>
+    <t>KBN_DONOR</t>
+  </si>
+  <si>
+    <t>SEX</t>
   </si>
   <si>
     <t>남</t>
@@ -28,10 +40,10 @@
     <t>여</t>
   </si>
   <si>
-    <t>출생연도</t>
-  </si>
-  <si>
-    <t>출생월</t>
+    <t>BIRTH_YEAR</t>
+  </si>
+  <si>
+    <t>BIRTH_MONTH</t>
   </si>
 </sst>
 </file>
@@ -363,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -374,37 +386,51 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2">
-        <v>10005</v>
+      <c r="A2" t="s">
+        <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>2001</v>
-      </c>
-      <c r="D2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3">
+        <v>10005</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>2001</v>
+      </c>
+      <c r="D3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4">
         <v>10008</v>
       </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3">
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4">
         <v>1993</v>
       </c>
-      <c r="D3">
+      <c r="D4">
         <v>2</v>
       </c>
     </row>

</xml_diff>